<commit_message>
[ENH] Modified instructions of module 2 and solved minor bugs.
</commit_message>
<xml_diff>
--- a/src/instructions/DVS_tracking_task_instructions.xlsx
+++ b/src/instructions/DVS_tracking_task_instructions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\siburmuin\src\begiBrainDemo\instructions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\begibraintool\src\instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{1D1147F3-3021-4AB8-A84A-106C411934A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66EC3D0D-6E93-4232-959E-6882526653A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>title</t>
   </si>
@@ -119,10 +119,13 @@
     <t>DVS TASK</t>
   </si>
   <si>
-    <t>En esta tarea debes seguir con la mirada el estímulo de color</t>
-  </si>
-  <si>
-    <t>Verás que se esconde del resto de puntos y que el movimiento del estímulo principal y del resto de bolas cambiará a lo largo del tiempo. Trata de seguirlo con la mayor precisión posible.</t>
+    <t>En esta tarea debes seguir con la mirada la bola de distinto color. Puede costar un poco encontrarla. Una vez la encuentres, no separes la mirada de la bola.</t>
+  </si>
+  <si>
+    <t>Verás que se esconde del resto de puntos y que el movimiento cambia. Trata de seguirlo con la mayor precisión posible.</t>
+  </si>
+  <si>
+    <t>Pulsa el botón central para empezar la prueba.</t>
   </si>
 </sst>
 </file>
@@ -552,6 +555,9 @@
       <c r="C2" t="s">
         <v>8</v>
       </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -680,18 +686,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -711,14 +717,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -731,4 +729,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>